<commit_message>
Castelnuovo: rendered walls of units 418 and 420 as Type D; façades and vulnerabilities in the knowledge record
The walls of unit 420 and the two upper storeys of unit 418 carried the Type A
and Type B materials although the survey classifies them as rendered (Type D).
The knowledge record now assigns the walls to the seven façades and records
their vulnerabilities, so the FMO rules derive behaviours and mechanisms.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/survey_data/castelnuovo/case.xlsx
+++ b/resources/survey_data/castelnuovo/case.xlsx
@@ -1232,7 +1232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1254,6 +1254,601 @@
       <c r="C1" s="1" t="inlineStr">
         <is>
           <t>evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417a</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DeformableFloors</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Timber floors alla romana documented for the aggregate as a whole (Section 8.2.3); no stiffening of the floors observed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417a</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopCurbstone</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Historic tuff masonry with timber floors and roofs; no curb beam visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417a</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateCurbstone</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>No curb beam visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417a</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopChains</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417a</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateChains</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417b</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DeformableFloors</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Timber floors alla romana documented for the aggregate as a whole (Section 8.2.3); no stiffening of the floors observed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417b</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopCurbstone</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Historic tuff masonry with timber floors and roofs; no curb beam visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417b</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateCurbstone</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>No curb beam visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417b</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopChains</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417b</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateChains</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417c</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>DeformableFloors</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Timber floors alla romana documented for the aggregate as a whole (Section 8.2.3); no stiffening of the floors observed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417c</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopCurbstone</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Historic tuff masonry with timber floors and roofs; no curb beam visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417c</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateCurbstone</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>No curb beam visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417c</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopChains</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Facade_417c</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateChains</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Facade_418a</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>DeformableFloors</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Timber floors alla romana documented for the aggregate as a whole (Section 8.2.3); no stiffening of the floors observed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Facade_418a</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopCurbstone</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Historic tuff masonry with timber floors and roofs; no curb beam visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Facade_418a</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateCurbstone</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>No curb beam visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Facade_418a</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopChains</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Facade_418a</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateChains</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Facade_418b</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>DeformableFloors</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Timber floors alla romana documented for the aggregate as a whole (Section 8.2.3); no stiffening of the floors observed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Facade_418b</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopCurbstone</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Historic tuff masonry with timber floors and roofs; no curb beam visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Facade_418b</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateCurbstone</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>No curb beam visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Facade_418b</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopChains</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Facade_418b</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateChains</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Facade_419</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>DeformableFloors</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Timber floors alla romana documented for the aggregate as a whole (Section 8.2.3); no stiffening of the floors observed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Facade_419</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopCurbstone</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Historic tuff masonry with timber floors and roofs; no curb beam visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Facade_419</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateCurbstone</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>No curb beam visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Facade_419</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopChains</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Facade_419</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateChains</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Facade_420</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>DeformableFloors</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Timber floors alla romana documented for the aggregate as a whole (Section 8.2.3); no stiffening of the floors observed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Facade_420</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopCurbstone</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Historic tuff masonry with timber floors and roofs; no curb beam visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Facade_420</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateCurbstone</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>No curb beam visible at the floor levels in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Facade_420</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfTopChains</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the top of the walls in the survey photographs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Facade_420</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>AbsenceOfIntermediateChains</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>No tie-rod anchor plates visible at the floor levels in the survey photographs.</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3933,11 @@
           <t>Tufelli_masonry_typeC</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>112HIUctr2yw5OqZgr3kla; 112HIUctr2yw5OqZgr3kXe; 112HIUctr2yw5OqZgr3kYs; 112HIUctr2yw5OqZgr3kaS; 3c8HC29$17vfNgcUAdeh3J; 3c8HC29$17vfNgcUAdeh3I; 3c8HC29$17vfNgcUAdeh3H; 3c8HC29$17vfNgcUAdeh3G; 1FujFrxrb7ouwnZEeyzKU0; 2HmFfYHsL2OPZKrO6tYf$1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3361,7 +3960,11 @@
           <t>Tufelli_masonry_typeD</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>3c8HC29$17vfNgcUAdeh01; 3c8HC29$17vfNgcUAdeh00; 3c8HC29$17vfNgcUAdeh07; 3c8HC29$17vfNgcUAdeh06; 0QfxonMDT2A8cO_M93$yye; 0QfxonMDT2A8cO_M93$yp8</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3384,7 +3987,11 @@
           <t>Tufelli_masonry_typeB</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2XzZEtRJH75fftbZbcqwO2; 2XzZEtRJH75fftbZbcqwH8; 2XzZEtRJH75fftbZbcqwJ5; 07H4IE3N17quz_RDvElapV</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3407,7 +4014,11 @@
           <t>Tufelli_masonry_typeB</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2XzZEtRJH75fftbZbcqwCR; 2XzZEtRJH75fftbZbcqwCB; 0CvVHHujLB8fkhpCAWbiT3; 1HfLPk$M547Aaac6ue3X37; 2tiNzAytfCwQOKJzMPcwjv</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3430,7 +4041,11 @@
           <t>Tufelli_masonry_typeD</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2XzZEtRJH75fftbZbcqwNS; 1HfLPk$M547Aaac6ue3X0L; 2QEzj1Im5478gG84LIeYU2; 2QEzj1Im5478gG84LIeYTv</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3453,7 +4068,11 @@
           <t>Tufelli_masonry_typeA</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>0GisCWViz2PeUrBi4wgVRW; 112HIUctr2yw5OqZgr3kPn; 112HIUctr2yw5OqZgr3kPe; 112HIUctr2yw5OqZgr3ksc; 0M1S9S_Qr3IPBMDqinoabk; 37gWW_uGL459BrbCF$MAq8; 2XzZEtRJH75fftbZbcqwY_; 2XzZEtRJH75fftbZbcqwZb; 2SDwapJ$z32OyuRGCv33co; 3_wR1BNVfAMeWWIaQS4y2L; 3_wR1BNVfAMeWWIaQS4ySL; 3_wR1BNVfAMeWWIaQS4yS9; 0F0gJxCaz6DgMK0q1JiO7L; 1aMTge6B9DK9$RHbrOwo4u</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3476,7 +4095,11 @@
           <t>Tufelli_masonry_typeD</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>0GisCWViz2PeUrBi4wgVUt; 0GisCWViz2PeUrBi4wgUZp; 0GisCWViz2PeUrBi4wgUdW; 0GisCWViz2PeUrBi4wgUa5; 112HIUctr2yw5OqZgr3kPo; 112HIUctr2yw5OqZgr3kPp; 112HIUctr2yw5OqZgr3kPi; 112HIUctr2yw5OqZgr3kPj; 112HIUctr2yw5OqZgr3kPf; 112HIUctr2yw5OqZgr3kPg; 112HIUctr2yw5OqZgr3kPh; 112HIUctr2yw5OqZgr3kPa</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Castelnuovo: top storeys of 417 and 418 in the masonry of the storeys below
The top storey of unit 417 is Type C and the two upper storeys of unit 418
are Type B, like the storeys below, instead of the rendered Type D: their
walls leave the Type D material association in final_example, example_clean
and castelnuovo_case, and in the knowledge record they move from facades
417b and 418b to 417a and 418a. Type D is now unit 420 only. Facades 417b
and 418b stay in the record, with no walls assigned.

The web export, the graph, the page and the volume materials of the
numerical model are regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/survey_data/castelnuovo/case.xlsx
+++ b/resources/survey_data/castelnuovo/case.xlsx
@@ -3935,7 +3935,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>112HIUctr2yw5OqZgr3kla; 112HIUctr2yw5OqZgr3kXe; 112HIUctr2yw5OqZgr3kYs; 112HIUctr2yw5OqZgr3kaS; 3c8HC29$17vfNgcUAdeh3J; 3c8HC29$17vfNgcUAdeh3I; 3c8HC29$17vfNgcUAdeh3H; 3c8HC29$17vfNgcUAdeh3G; 1FujFrxrb7ouwnZEeyzKU0; 2HmFfYHsL2OPZKrO6tYf$1</t>
+          <t>112HIUctr2yw5OqZgr3kla; 112HIUctr2yw5OqZgr3kXe; 112HIUctr2yw5OqZgr3kYs; 112HIUctr2yw5OqZgr3kaS; 3c8HC29$17vfNgcUAdeh3J; 3c8HC29$17vfNgcUAdeh3I; 3c8HC29$17vfNgcUAdeh3H; 3c8HC29$17vfNgcUAdeh3G; 1FujFrxrb7ouwnZEeyzKU0; 2HmFfYHsL2OPZKrO6tYf$1; 3c8HC29$17vfNgcUAdeh01; 3c8HC29$17vfNgcUAdeh00; 3c8HC29$17vfNgcUAdeh07; 3c8HC29$17vfNgcUAdeh06; 0QfxonMDT2A8cO_M93$yye; 0QfxonMDT2A8cO_M93$yp8</t>
         </is>
       </c>
     </row>
@@ -3960,11 +3960,7 @@
           <t>Tufelli_masonry_typeD</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>3c8HC29$17vfNgcUAdeh01; 3c8HC29$17vfNgcUAdeh00; 3c8HC29$17vfNgcUAdeh07; 3c8HC29$17vfNgcUAdeh06; 0QfxonMDT2A8cO_M93$yye; 0QfxonMDT2A8cO_M93$yp8</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4016,7 +4012,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2XzZEtRJH75fftbZbcqwCR; 2XzZEtRJH75fftbZbcqwCB; 0CvVHHujLB8fkhpCAWbiT3; 1HfLPk$M547Aaac6ue3X37; 2tiNzAytfCwQOKJzMPcwjv</t>
+          <t>2XzZEtRJH75fftbZbcqwCR; 2XzZEtRJH75fftbZbcqwCB; 0CvVHHujLB8fkhpCAWbiT3; 1HfLPk$M547Aaac6ue3X37; 2tiNzAytfCwQOKJzMPcwjv; 2XzZEtRJH75fftbZbcqwNS; 1HfLPk$M547Aaac6ue3X0L; 2QEzj1Im5478gG84LIeYU2; 2QEzj1Im5478gG84LIeYTv</t>
         </is>
       </c>
     </row>
@@ -4041,11 +4037,7 @@
           <t>Tufelli_masonry_typeD</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>2XzZEtRJH75fftbZbcqwNS; 1HfLPk$M547Aaac6ue3X0L; 2QEzj1Im5478gG84LIeYU2; 2QEzj1Im5478gG84LIeYTv</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Castelnuovo: units numbered from the right end; Type B walls are rendered (Type D)
The units were numbered from the wrong end of the aggregate. From the south
end they are 417, 418, 419 and 420, and the knowledge record now assigns the
walls accordingly: unit 417 to facade 417a, 418 to 418a, 419 and 420 to their
facades. The masonry types are those of the BIM model, except that every wall
modelled as Type B is rendered and takes Type D: 417 D, 418 A, 419 D, 420 C.
Facades 417b, 417c and 418b stay in the record with no walls.

The web export, the graph, the page, the volume materials and the case-study
pages of the documentation are regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/survey_data/castelnuovo/case.xlsx
+++ b/resources/survey_data/castelnuovo/case.xlsx
@@ -3930,12 +3930,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Tufelli_masonry_typeC</t>
+          <t>Tufelli_masonry_typeD</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>112HIUctr2yw5OqZgr3kla; 112HIUctr2yw5OqZgr3kXe; 112HIUctr2yw5OqZgr3kYs; 112HIUctr2yw5OqZgr3kaS; 3c8HC29$17vfNgcUAdeh3J; 3c8HC29$17vfNgcUAdeh3I; 3c8HC29$17vfNgcUAdeh3H; 3c8HC29$17vfNgcUAdeh3G; 1FujFrxrb7ouwnZEeyzKU0; 2HmFfYHsL2OPZKrO6tYf$1; 3c8HC29$17vfNgcUAdeh01; 3c8HC29$17vfNgcUAdeh00; 3c8HC29$17vfNgcUAdeh07; 3c8HC29$17vfNgcUAdeh06; 0QfxonMDT2A8cO_M93$yye; 0QfxonMDT2A8cO_M93$yp8</t>
+          <t>0GisCWViz2PeUrBi4wgVUt; 0GisCWViz2PeUrBi4wgUZp; 0GisCWViz2PeUrBi4wgUdW; 0GisCWViz2PeUrBi4wgUa5; 112HIUctr2yw5OqZgr3kPo; 112HIUctr2yw5OqZgr3kPp; 112HIUctr2yw5OqZgr3kPi; 112HIUctr2yw5OqZgr3kPj; 112HIUctr2yw5OqZgr3kPf; 112HIUctr2yw5OqZgr3kPg; 112HIUctr2yw5OqZgr3kPh; 112HIUctr2yw5OqZgr3kPa</t>
         </is>
       </c>
     </row>
@@ -3980,14 +3980,10 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Tufelli_masonry_typeB</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>2XzZEtRJH75fftbZbcqwO2; 2XzZEtRJH75fftbZbcqwH8; 2XzZEtRJH75fftbZbcqwJ5; 07H4IE3N17quz_RDvElapV</t>
-        </is>
-      </c>
+          <t>Tufelli_masonry_typeD</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4007,12 +4003,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Tufelli_masonry_typeB</t>
+          <t>Tufelli_masonry_typeA</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2XzZEtRJH75fftbZbcqwCR; 2XzZEtRJH75fftbZbcqwCB; 0CvVHHujLB8fkhpCAWbiT3; 1HfLPk$M547Aaac6ue3X37; 2tiNzAytfCwQOKJzMPcwjv; 2XzZEtRJH75fftbZbcqwNS; 1HfLPk$M547Aaac6ue3X0L; 2QEzj1Im5478gG84LIeYU2; 2QEzj1Im5478gG84LIeYTv</t>
+          <t>0GisCWViz2PeUrBi4wgVRW; 112HIUctr2yw5OqZgr3kPn; 112HIUctr2yw5OqZgr3kPe; 112HIUctr2yw5OqZgr3ksc; 0M1S9S_Qr3IPBMDqinoabk; 37gWW_uGL459BrbCF$MAq8; 2XzZEtRJH75fftbZbcqwY_; 2XzZEtRJH75fftbZbcqwZb; 2SDwapJ$z32OyuRGCv33co; 3_wR1BNVfAMeWWIaQS4y2L; 3_wR1BNVfAMeWWIaQS4ySL; 3_wR1BNVfAMeWWIaQS4yS9; 0F0gJxCaz6DgMK0q1JiO7L; 1aMTge6B9DK9$RHbrOwo4u</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4030,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Tufelli_masonry_typeD</t>
+          <t>Tufelli_masonry_typeA</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
@@ -4057,12 +4053,12 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Tufelli_masonry_typeA</t>
+          <t>Tufelli_masonry_typeD</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>0GisCWViz2PeUrBi4wgVRW; 112HIUctr2yw5OqZgr3kPn; 112HIUctr2yw5OqZgr3kPe; 112HIUctr2yw5OqZgr3ksc; 0M1S9S_Qr3IPBMDqinoabk; 37gWW_uGL459BrbCF$MAq8; 2XzZEtRJH75fftbZbcqwY_; 2XzZEtRJH75fftbZbcqwZb; 2SDwapJ$z32OyuRGCv33co; 3_wR1BNVfAMeWWIaQS4y2L; 3_wR1BNVfAMeWWIaQS4ySL; 3_wR1BNVfAMeWWIaQS4yS9; 0F0gJxCaz6DgMK0q1JiO7L; 1aMTge6B9DK9$RHbrOwo4u</t>
+          <t>2XzZEtRJH75fftbZbcqwCR; 2XzZEtRJH75fftbZbcqwCB; 0CvVHHujLB8fkhpCAWbiT3; 1HfLPk$M547Aaac6ue3X37; 2tiNzAytfCwQOKJzMPcwjv; 2XzZEtRJH75fftbZbcqwNS; 1HfLPk$M547Aaac6ue3X0L; 2QEzj1Im5478gG84LIeYU2; 2QEzj1Im5478gG84LIeYTv; 2XzZEtRJH75fftbZbcqwO2; 2XzZEtRJH75fftbZbcqwH8; 2XzZEtRJH75fftbZbcqwJ5; 07H4IE3N17quz_RDvElapV</t>
         </is>
       </c>
     </row>
@@ -4084,12 +4080,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Tufelli_masonry_typeD</t>
+          <t>Tufelli_masonry_typeC</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>0GisCWViz2PeUrBi4wgVUt; 0GisCWViz2PeUrBi4wgUZp; 0GisCWViz2PeUrBi4wgUdW; 0GisCWViz2PeUrBi4wgUa5; 112HIUctr2yw5OqZgr3kPo; 112HIUctr2yw5OqZgr3kPp; 112HIUctr2yw5OqZgr3kPi; 112HIUctr2yw5OqZgr3kPj; 112HIUctr2yw5OqZgr3kPf; 112HIUctr2yw5OqZgr3kPg; 112HIUctr2yw5OqZgr3kPh; 112HIUctr2yw5OqZgr3kPa</t>
+          <t>112HIUctr2yw5OqZgr3kla; 112HIUctr2yw5OqZgr3kXe; 112HIUctr2yw5OqZgr3kYs; 112HIUctr2yw5OqZgr3kaS; 3c8HC29$17vfNgcUAdeh3J; 3c8HC29$17vfNgcUAdeh3I; 3c8HC29$17vfNgcUAdeh3H; 3c8HC29$17vfNgcUAdeh3G; 1FujFrxrb7ouwnZEeyzKU0; 2HmFfYHsL2OPZKrO6tYf$1; 3c8HC29$17vfNgcUAdeh01; 3c8HC29$17vfNgcUAdeh00; 3c8HC29$17vfNgcUAdeh07; 3c8HC29$17vfNgcUAdeh06; 0QfxonMDT2A8cO_M93$yye; 0QfxonMDT2A8cO_M93$yp8</t>
         </is>
       </c>
     </row>

</xml_diff>